<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-10-26.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-10-26.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-10-26.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L49"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -741,32 +741,118 @@
         <v>6</v>
       </c>
       <c r="C37" t="str">
-        <v>870_干花安娜绣球红_undefined_undefined_1bunch</v>
+        <v>633_干花安娜深红_undefined_undefined_1stem</v>
+      </c>
+      <c r="F37" t="str">
+        <v>50</v>
       </c>
     </row>
     <row r="38">
       <c r="C38" t="str">
         <v>636_干花大叶白_undefined_undefined_1stem</v>
       </c>
+      <c r="F38" t="str">
+        <v>50</v>
+      </c>
     </row>
     <row r="39">
       <c r="C39" t="str">
         <v>635_干花安娜白_undefined_undefined_1stem</v>
       </c>
+      <c r="F39" t="str">
+        <v>15</v>
+      </c>
     </row>
     <row r="40">
       <c r="C40" t="str">
         <v>635_干花安娜白_undefined_undefined_1stem</v>
       </c>
+      <c r="F40" t="str">
+        <v>15</v>
+      </c>
     </row>
     <row r="41">
       <c r="C41" t="str">
         <v>636_干花大叶白_undefined_undefined_1stem</v>
       </c>
+      <c r="F41" t="str">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>7</v>
+      </c>
+      <c r="C42" t="str">
+        <v>47_拉丝玫红_Spider Dark Pink_Gerbera L._20stems</v>
+      </c>
+      <c r="F42" t="str">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" t="str">
+        <v>480_蝴蝶洋牡丹红_butterfly  Ranunculus_undefined_1bunch</v>
+      </c>
+      <c r="F43" t="str">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="C44" t="str" xml:space="preserve">
+        <v xml:space="preserve">553_嘉兰百合
+multi-colors_ gloriosa_undefined_1bunch</v>
+      </c>
+      <c r="F44" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="C45" t="str">
+        <v>649_洋牡丹樱花粉_undefined_undefined_1bunch</v>
+      </c>
+      <c r="F45" t="str">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="C46" t="str">
+        <v>643_巧克力秋英_undefined_undefined_1bunch</v>
+      </c>
+      <c r="F46" t="str">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" t="str">
+        <v>300_白星_White Gypso_ gypsophila_1kg</v>
+      </c>
+      <c r="F47" t="str">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>8</v>
+      </c>
+      <c r="C48" t="str">
+        <v>633_干花安娜深红_undefined_undefined_1stem</v>
+      </c>
+      <c r="F48" t="str">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49" t="str">
+        <v>862_干花黄金球白_undefined_undefined_1bunch</v>
+      </c>
+      <c r="F49" t="str">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L49"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -821,7 +907,7 @@
         <v>0.00</v>
       </c>
       <c r="G2" t="str">
-        <v>058512101255205102020365565552855171015128101616252000000</v>
+        <v>05851210125520510202036556555285517101512810161625205050151515205255103010</v>
       </c>
     </row>
   </sheetData>

</xml_diff>